<commit_message>
Model recalibration based on new project data on HIV DR
- Revised HIV DR calibration data based on the project - August 12th data
- Revised calibrations
- Revised the Bayesian calibration vector to incorporate the new data
</commit_message>
<xml_diff>
--- a/output/diagnostics/Bayesian_parameter(results).xlsx
+++ b/output/diagnostics/Bayesian_parameter(results).xlsx
@@ -482,31 +482,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.975</v>
+        <v>0.878</v>
       </c>
       <c r="C2" t="n">
-        <v>0.207</v>
+        <v>0.18</v>
       </c>
       <c r="D2" t="n">
-        <v>0.593</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>1.327</v>
+        <v>1.206</v>
       </c>
       <c r="F2" t="n">
         <v>0.006</v>
       </c>
       <c r="G2" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="H2" t="n">
-        <v>1033</v>
+        <v>880</v>
       </c>
       <c r="I2" t="n">
-        <v>915</v>
+        <v>783</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="3">
@@ -516,16 +516,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.486</v>
+        <v>0.489</v>
       </c>
       <c r="C3" t="n">
-        <v>0.163</v>
+        <v>0.172</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2</v>
+        <v>0.208</v>
       </c>
       <c r="E3" t="n">
-        <v>0.785</v>
+        <v>0.831</v>
       </c>
       <c r="F3" t="n">
         <v>0.004</v>
@@ -534,10 +534,10 @@
         <v>0.005</v>
       </c>
       <c r="H3" t="n">
-        <v>1383</v>
+        <v>1400</v>
       </c>
       <c r="I3" t="n">
-        <v>768</v>
+        <v>629</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -550,28 +550,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.509</v>
+        <v>0.492</v>
       </c>
       <c r="C4" t="n">
-        <v>0.16</v>
+        <v>0.151</v>
       </c>
       <c r="D4" t="n">
-        <v>0.239</v>
+        <v>0.246</v>
       </c>
       <c r="E4" t="n">
-        <v>0.792</v>
+        <v>0.772</v>
       </c>
       <c r="F4" t="n">
         <v>0.005</v>
       </c>
       <c r="G4" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="H4" t="n">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="I4" t="n">
-        <v>822</v>
+        <v>635</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -590,7 +590,7 @@
         <v>0.014</v>
       </c>
       <c r="D5" t="n">
-        <v>0.092</v>
+        <v>0.094</v>
       </c>
       <c r="E5" t="n">
         <v>0.146</v>
@@ -602,10 +602,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>540</v>
+        <v>503</v>
       </c>
       <c r="I5" t="n">
-        <v>583</v>
+        <v>699</v>
       </c>
       <c r="J5" t="n">
         <v>1.01</v>
@@ -618,13 +618,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="D6" t="n">
-        <v>0.022</v>
+        <v>0.03</v>
       </c>
       <c r="E6" t="n">
         <v>0.151</v>
@@ -636,13 +636,13 @@
         <v>0.001</v>
       </c>
       <c r="H6" t="n">
-        <v>1329</v>
+        <v>1463</v>
       </c>
       <c r="I6" t="n">
-        <v>777</v>
+        <v>821</v>
       </c>
       <c r="J6" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -652,28 +652,28 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.271</v>
+        <v>1.12</v>
       </c>
       <c r="C7" t="n">
-        <v>0.448</v>
+        <v>0.401</v>
       </c>
       <c r="D7" t="n">
-        <v>0.581</v>
+        <v>0.445</v>
       </c>
       <c r="E7" t="n">
-        <v>2.135</v>
+        <v>1.804</v>
       </c>
       <c r="F7" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="G7" t="n">
-        <v>0.014</v>
+        <v>0.016</v>
       </c>
       <c r="H7" t="n">
-        <v>1193</v>
+        <v>1247</v>
       </c>
       <c r="I7" t="n">
-        <v>915</v>
+        <v>850</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -686,16 +686,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="E8" t="n">
-        <v>0.059</v>
+        <v>0.058</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -704,13 +704,13 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>1132</v>
+        <v>1006</v>
       </c>
       <c r="I8" t="n">
-        <v>782</v>
+        <v>876</v>
       </c>
       <c r="J8" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.256</v>
+        <v>0.253</v>
       </c>
       <c r="C9" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="D9" t="n">
-        <v>0.161</v>
+        <v>0.151</v>
       </c>
       <c r="E9" t="n">
-        <v>0.368</v>
+        <v>0.354</v>
       </c>
       <c r="F9" t="n">
         <v>0.001</v>
@@ -738,13 +738,13 @@
         <v>0.002</v>
       </c>
       <c r="H9" t="n">
-        <v>1509</v>
+        <v>1379</v>
       </c>
       <c r="I9" t="n">
-        <v>646</v>
+        <v>788</v>
       </c>
       <c r="J9" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -760,22 +760,22 @@
         <v>0.074</v>
       </c>
       <c r="D10" t="n">
-        <v>0.218</v>
+        <v>0.227</v>
       </c>
       <c r="E10" t="n">
-        <v>0.487</v>
+        <v>0.507</v>
       </c>
       <c r="F10" t="n">
         <v>0.002</v>
       </c>
       <c r="G10" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="H10" t="n">
-        <v>1755</v>
+        <v>1600</v>
       </c>
       <c r="I10" t="n">
-        <v>784</v>
+        <v>760</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
@@ -794,7 +794,7 @@
         <v>0.005</v>
       </c>
       <c r="D11" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E11" t="n">
         <v>0.025</v>
@@ -806,13 +806,13 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>495</v>
+        <v>458</v>
       </c>
       <c r="I11" t="n">
-        <v>671</v>
+        <v>611</v>
       </c>
       <c r="J11" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -822,28 +822,28 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.759</v>
+        <v>0.742</v>
       </c>
       <c r="C12" t="n">
-        <v>0.258</v>
+        <v>0.262</v>
       </c>
       <c r="D12" t="n">
-        <v>0.322</v>
+        <v>0.31</v>
       </c>
       <c r="E12" t="n">
-        <v>1.238</v>
+        <v>1.215</v>
       </c>
       <c r="F12" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>1752</v>
+        <v>1279</v>
       </c>
       <c r="I12" t="n">
-        <v>714</v>
+        <v>726</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -856,28 +856,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.175</v>
+        <v>0.176</v>
       </c>
       <c r="C13" t="n">
-        <v>0.093</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="E13" t="n">
-        <v>0.354</v>
+        <v>0.332</v>
       </c>
       <c r="F13" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="G13" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="H13" t="n">
-        <v>1941</v>
+        <v>1211</v>
       </c>
       <c r="I13" t="n">
-        <v>753</v>
+        <v>651</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -890,28 +890,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.525</v>
+        <v>1.48</v>
       </c>
       <c r="C14" t="n">
-        <v>0.628</v>
+        <v>0.636</v>
       </c>
       <c r="D14" t="n">
-        <v>0.36</v>
+        <v>0.431</v>
       </c>
       <c r="E14" t="n">
-        <v>2.626</v>
+        <v>2.65</v>
       </c>
       <c r="F14" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="G14" t="n">
-        <v>0.021</v>
+        <v>0.02</v>
       </c>
       <c r="H14" t="n">
-        <v>1420</v>
+        <v>773</v>
       </c>
       <c r="I14" t="n">
-        <v>809</v>
+        <v>537</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
@@ -927,28 +927,28 @@
         <v>2.435</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.545</v>
       </c>
       <c r="D15" t="n">
-        <v>1.372</v>
+        <v>1.537</v>
       </c>
       <c r="E15" t="n">
-        <v>3.39</v>
+        <v>3.487</v>
       </c>
       <c r="F15" t="n">
         <v>0.014</v>
       </c>
       <c r="G15" t="n">
-        <v>0.022</v>
+        <v>0.018</v>
       </c>
       <c r="H15" t="n">
-        <v>1578</v>
+        <v>1582</v>
       </c>
       <c r="I15" t="n">
-        <v>428</v>
+        <v>605</v>
       </c>
       <c r="J15" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -958,28 +958,28 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.18</v>
+        <v>3.31</v>
       </c>
       <c r="C16" t="n">
-        <v>1.159</v>
+        <v>1.25</v>
       </c>
       <c r="D16" t="n">
-        <v>1.5</v>
+        <v>1.518</v>
       </c>
       <c r="E16" t="n">
-        <v>5.267</v>
+        <v>5.531</v>
       </c>
       <c r="F16" t="n">
-        <v>0.03</v>
+        <v>0.047</v>
       </c>
       <c r="G16" t="n">
-        <v>0.03</v>
+        <v>0.031</v>
       </c>
       <c r="H16" t="n">
-        <v>1532</v>
+        <v>803</v>
       </c>
       <c r="I16" t="n">
-        <v>553</v>
+        <v>412</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
@@ -992,31 +992,31 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.578</v>
+        <v>0.572</v>
       </c>
       <c r="C17" t="n">
-        <v>0.314</v>
+        <v>0.318</v>
       </c>
       <c r="D17" t="n">
-        <v>0.076</v>
+        <v>0.043</v>
       </c>
       <c r="E17" t="n">
-        <v>1.135</v>
+        <v>1.099</v>
       </c>
       <c r="F17" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="G17" t="n">
         <v>0.012</v>
       </c>
-      <c r="G17" t="n">
-        <v>0.01</v>
-      </c>
       <c r="H17" t="n">
-        <v>653</v>
+        <v>493</v>
       </c>
       <c r="I17" t="n">
-        <v>709</v>
+        <v>555</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="18">
@@ -1029,25 +1029,25 @@
         <v>0.587</v>
       </c>
       <c r="C18" t="n">
-        <v>0.273</v>
+        <v>0.311</v>
       </c>
       <c r="D18" t="n">
-        <v>0.16</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>1.13</v>
+        <v>1.158</v>
       </c>
       <c r="F18" t="n">
         <v>0.008</v>
       </c>
       <c r="G18" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="H18" t="n">
-        <v>1154</v>
+        <v>1253</v>
       </c>
       <c r="I18" t="n">
-        <v>752</v>
+        <v>533</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
@@ -1060,28 +1060,28 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>22.745</v>
+        <v>22.737</v>
       </c>
       <c r="C19" t="n">
         <v>1.745</v>
       </c>
       <c r="D19" t="n">
-        <v>20.022</v>
+        <v>20.031</v>
       </c>
       <c r="E19" t="n">
-        <v>25.623</v>
+        <v>25.514</v>
       </c>
       <c r="F19" t="n">
-        <v>0.045</v>
+        <v>0.043</v>
       </c>
       <c r="G19" t="n">
-        <v>0.036</v>
+        <v>0.039</v>
       </c>
       <c r="H19" t="n">
-        <v>1282</v>
+        <v>1445</v>
       </c>
       <c r="I19" t="n">
-        <v>599</v>
+        <v>652</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -1094,31 +1094,31 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.66</v>
+        <v>0.672</v>
       </c>
       <c r="C20" t="n">
-        <v>0.201</v>
+        <v>0.196</v>
       </c>
       <c r="D20" t="n">
-        <v>0.272</v>
+        <v>0.315</v>
       </c>
       <c r="E20" t="n">
-        <v>0.984</v>
+        <v>1.005</v>
       </c>
       <c r="F20" t="n">
         <v>0.005</v>
       </c>
       <c r="G20" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
       <c r="H20" t="n">
-        <v>1608</v>
+        <v>1342</v>
       </c>
       <c r="I20" t="n">
-        <v>473</v>
+        <v>651</v>
       </c>
       <c r="J20" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1128,31 +1128,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.186</v>
+        <v>0.174</v>
       </c>
       <c r="C21" t="n">
-        <v>0.058</v>
+        <v>0.049</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1</v>
+        <v>0.096</v>
       </c>
       <c r="E21" t="n">
-        <v>0.284</v>
+        <v>0.257</v>
       </c>
       <c r="F21" t="n">
         <v>0.002</v>
       </c>
       <c r="G21" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="H21" t="n">
-        <v>766</v>
+        <v>783</v>
       </c>
       <c r="I21" t="n">
-        <v>749</v>
+        <v>655</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="22">
@@ -1171,7 +1171,7 @@
         <v>0.042</v>
       </c>
       <c r="E22" t="n">
-        <v>0.06</v>
+        <v>0.059</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1180,13 +1180,13 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>511</v>
+        <v>446</v>
       </c>
       <c r="I22" t="n">
-        <v>730</v>
+        <v>641</v>
       </c>
       <c r="J22" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1196,31 +1196,31 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="C23" t="n">
-        <v>0.133</v>
+        <v>0.127</v>
       </c>
       <c r="D23" t="n">
-        <v>0.457</v>
+        <v>0.454</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="F23" t="n">
         <v>0.003</v>
       </c>
       <c r="G23" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="H23" t="n">
-        <v>1541</v>
+        <v>1242</v>
       </c>
       <c r="I23" t="n">
-        <v>621</v>
+        <v>631</v>
       </c>
       <c r="J23" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1233,13 +1233,13 @@
         <v>0.05</v>
       </c>
       <c r="C24" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="D24" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="E24" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.082</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1248,13 +1248,13 @@
         <v>0.001</v>
       </c>
       <c r="H24" t="n">
-        <v>1674</v>
+        <v>1512</v>
       </c>
       <c r="I24" t="n">
-        <v>603</v>
+        <v>366</v>
       </c>
       <c r="J24" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1264,16 +1264,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="C25" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="D25" t="n">
         <v>0.022</v>
       </c>
       <c r="E25" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1282,13 +1282,13 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1774</v>
+        <v>1154</v>
       </c>
       <c r="I25" t="n">
-        <v>818</v>
+        <v>652</v>
       </c>
       <c r="J25" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1304,7 +1304,7 @@
         <v>0.006</v>
       </c>
       <c r="D26" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="E26" t="n">
         <v>0.034</v>
@@ -1316,10 +1316,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1947</v>
+        <v>1862</v>
       </c>
       <c r="I26" t="n">
-        <v>824</v>
+        <v>780</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
@@ -1332,31 +1332,31 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3.158</v>
+        <v>3.201</v>
       </c>
       <c r="C27" t="n">
-        <v>0.629</v>
+        <v>0.67</v>
       </c>
       <c r="D27" t="n">
-        <v>2.035</v>
+        <v>2.132</v>
       </c>
       <c r="E27" t="n">
-        <v>4.31</v>
+        <v>4.607</v>
       </c>
       <c r="F27" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="G27" t="n">
         <v>0.025</v>
       </c>
       <c r="H27" t="n">
-        <v>1316</v>
+        <v>1715</v>
       </c>
       <c r="I27" t="n">
-        <v>757</v>
+        <v>665</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="28">
@@ -1366,16 +1366,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.077</v>
+        <v>0.076</v>
       </c>
       <c r="C28" t="n">
-        <v>0.02</v>
+        <v>0.019</v>
       </c>
       <c r="D28" t="n">
         <v>0.042</v>
       </c>
       <c r="E28" t="n">
-        <v>0.115</v>
+        <v>0.112</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1384,10 +1384,10 @@
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>2528</v>
+        <v>1455</v>
       </c>
       <c r="I28" t="n">
-        <v>898</v>
+        <v>651</v>
       </c>
       <c r="J28" t="n">
         <v>1.01</v>
@@ -1400,28 +1400,28 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.222</v>
+        <v>0.22</v>
       </c>
       <c r="C29" t="n">
-        <v>0.062</v>
+        <v>0.06</v>
       </c>
       <c r="D29" t="n">
-        <v>0.108</v>
+        <v>0.115</v>
       </c>
       <c r="E29" t="n">
-        <v>0.334</v>
+        <v>0.328</v>
       </c>
       <c r="F29" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="G29" t="n">
         <v>0.002</v>
       </c>
       <c r="H29" t="n">
-        <v>1356</v>
+        <v>1823</v>
       </c>
       <c r="I29" t="n">
-        <v>632</v>
+        <v>906</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -1434,28 +1434,28 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.07</v>
+        <v>1.064</v>
       </c>
       <c r="C30" t="n">
-        <v>0.221</v>
+        <v>0.206</v>
       </c>
       <c r="D30" t="n">
-        <v>0.707</v>
+        <v>0.709</v>
       </c>
       <c r="E30" t="n">
-        <v>1.499</v>
+        <v>1.461</v>
       </c>
       <c r="F30" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G30" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="H30" t="n">
-        <v>1511</v>
+        <v>1678</v>
       </c>
       <c r="I30" t="n">
-        <v>587</v>
+        <v>731</v>
       </c>
       <c r="J30" t="n">
         <v>1</v>
@@ -1486,13 +1486,13 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1319</v>
+        <v>907</v>
       </c>
       <c r="I31" t="n">
-        <v>486</v>
+        <v>524</v>
       </c>
       <c r="J31" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1502,31 +1502,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>20939.622</v>
+        <v>27117.895</v>
       </c>
       <c r="C32" t="n">
-        <v>80446.257</v>
+        <v>97345.39999999999</v>
       </c>
       <c r="D32" t="n">
-        <v>562.1799999999999</v>
+        <v>650.027</v>
       </c>
       <c r="E32" t="n">
-        <v>66283.069</v>
+        <v>80828.74400000001</v>
       </c>
       <c r="F32" t="n">
-        <v>2836.893</v>
+        <v>4210.557</v>
       </c>
       <c r="G32" t="n">
-        <v>23284.58</v>
+        <v>19440.509</v>
       </c>
       <c r="H32" t="n">
-        <v>1319</v>
+        <v>907</v>
       </c>
       <c r="I32" t="n">
-        <v>486</v>
+        <v>524</v>
       </c>
       <c r="J32" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>